<commit_message>
updated ux lite score equation
</commit_message>
<xml_diff>
--- a/pendo-pipeline/data/config/xm_pendo_app_registry.xlsx
+++ b/pendo-pipeline/data/config/xm_pendo_app_registry.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/HC28ZB2/Library/CloudStorage/OneDrive-TheHomeDepot/Code/Python-Projects/pendo-pipeline/data/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedrive.homedepot.com/personal/nicole_erickson_homedepot_com/Documents/Code/Python-Projects/pendo-pipeline/data/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083CABC0-F403-EA48-9013-D287C28D7E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB4B1954-05C8-C942-AC6B-FAD499F43383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="520" windowWidth="22940" windowHeight="12760" xr2:uid="{76643C02-4F01-0E48-A18E-EEF1B4F036BD}"/>
+    <workbookView xWindow="0" yWindow="540" windowWidth="22940" windowHeight="12640" xr2:uid="{76643C02-4F01-0E48-A18E-EEF1B4F036BD}"/>
   </bookViews>
   <sheets>
-    <sheet name="xm_pendo_app_registry-write" sheetId="1" r:id="rId1"/>
+    <sheet name="xm_pendo_app_registry" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="162">
   <si>
     <t xml:space="preserve">Store </t>
   </si>
@@ -86,9 +86,6 @@
     <t>pendo_app_name</t>
   </si>
   <si>
-    <t>EFS</t>
-  </si>
-  <si>
     <t>ONT</t>
   </si>
   <si>
@@ -443,12 +440,6 @@
     <t>Store Order Fufillment (OFA)</t>
   </si>
   <si>
-    <t>Engineered Flow Schedule (EFS)</t>
-  </si>
-  <si>
-    <t>Engineered Flow Schedule</t>
-  </si>
-  <si>
     <t>ProAssist</t>
   </si>
   <si>
@@ -525,6 +516,9 @@
   </si>
   <si>
     <t>Orderability</t>
+  </si>
+  <si>
+    <t>Parm Light</t>
   </si>
 </sst>
 </file>
@@ -1116,6 +1110,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{16E8A365-EABF-9D4A-A256-86868040FC3B}" name="Table1" displayName="Table1" ref="A1:M56" totalsRowShown="0">
   <autoFilter ref="A1:M56" xr:uid="{16E8A365-EABF-9D4A-A256-86868040FC3B}"/>
@@ -1459,7 +1457,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE2CE3F0-7A6A-D042-BAD8-7639F1F4D7EA}">
   <dimension ref="A1:M58"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="1" customWidth="1"/>
@@ -1481,40 +1479,40 @@
         <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
@@ -1522,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>13</v>
@@ -1531,22 +1529,22 @@
         <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M2" s="1"/>
     </row>
@@ -1555,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>13</v>
@@ -1564,25 +1562,25 @@
         <v>5</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K3" s="2">
         <v>45959</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="M3" s="1"/>
     </row>
@@ -1591,7 +1589,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>13</v>
@@ -1600,7 +1598,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>4</v>
@@ -1615,7 +1613,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -1624,7 +1622,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>4</v>
@@ -1639,7 +1637,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>13</v>
@@ -1666,7 +1664,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
@@ -1675,13 +1673,13 @@
         <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>1</v>
@@ -1690,7 +1688,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M7" s="1"/>
     </row>
@@ -1699,7 +1697,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>13</v>
@@ -1708,13 +1706,13 @@
         <v>5</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>1</v>
@@ -1723,7 +1721,7 @@
         <v>1</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M8" s="1"/>
     </row>
@@ -1732,7 +1730,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -1741,19 +1739,19 @@
         <v>5</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M9" s="1"/>
     </row>
@@ -1762,7 +1760,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>13</v>
@@ -1771,13 +1769,13 @@
         <v>6</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>1</v>
@@ -1786,7 +1784,7 @@
         <v>1</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M10" s="1"/>
     </row>
@@ -1795,7 +1793,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>12</v>
@@ -1804,13 +1802,13 @@
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>1</v>
@@ -1819,7 +1817,7 @@
         <v>1</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M11" s="1"/>
     </row>
@@ -1828,7 +1826,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>13</v>
@@ -1837,13 +1835,13 @@
         <v>5</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>1</v>
@@ -1852,7 +1850,7 @@
         <v>1</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M12" s="1"/>
     </row>
@@ -1861,7 +1859,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>12</v>
@@ -1870,19 +1868,19 @@
         <v>5</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M13" s="1"/>
     </row>
@@ -1891,7 +1889,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>13</v>
@@ -1900,19 +1898,19 @@
         <v>7</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M14" s="1"/>
     </row>
@@ -1921,7 +1919,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>13</v>
@@ -1930,19 +1928,19 @@
         <v>7</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M15" s="1"/>
     </row>
@@ -1951,7 +1949,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>13</v>
@@ -1960,13 +1958,13 @@
         <v>7</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>1</v>
@@ -1975,7 +1973,7 @@
         <v>1</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M16" s="1"/>
     </row>
@@ -1984,7 +1982,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>13</v>
@@ -1993,13 +1991,13 @@
         <v>7</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>1</v>
@@ -2008,7 +2006,7 @@
         <v>1</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M17" s="1"/>
     </row>
@@ -2017,7 +2015,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>13</v>
@@ -2026,19 +2024,19 @@
         <v>6</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>17</v>
+        <v>161</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M18" s="1"/>
     </row>
@@ -2047,7 +2045,7 @@
         <v>1</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>12</v>
@@ -2056,13 +2054,13 @@
         <v>0</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>1</v>
@@ -2071,7 +2069,7 @@
         <v>1</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M19" s="1"/>
     </row>
@@ -2080,7 +2078,7 @@
         <v>1</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>12</v>
@@ -2089,13 +2087,13 @@
         <v>0</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>1</v>
@@ -2104,7 +2102,7 @@
         <v>1</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M20" s="1"/>
     </row>
@@ -2113,7 +2111,7 @@
         <v>1</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>12</v>
@@ -2122,13 +2120,13 @@
         <v>2</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>1</v>
@@ -2140,7 +2138,7 @@
         <v>45957</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M21" s="1"/>
     </row>
@@ -2149,7 +2147,7 @@
         <v>1</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>12</v>
@@ -2158,13 +2156,13 @@
         <v>10</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>1</v>
@@ -2173,7 +2171,7 @@
         <v>1</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M22" s="1"/>
     </row>
@@ -2182,7 +2180,7 @@
         <v>1</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>13</v>
@@ -2191,13 +2189,13 @@
         <v>7</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>1</v>
@@ -2206,7 +2204,7 @@
         <v>1</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M23" s="1"/>
     </row>
@@ -2215,7 +2213,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>13</v>
@@ -2224,13 +2222,13 @@
         <v>7</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>1</v>
@@ -2239,7 +2237,7 @@
         <v>1</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M24" s="1"/>
     </row>
@@ -2248,7 +2246,7 @@
         <v>1</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>13</v>
@@ -2257,19 +2255,19 @@
         <v>5</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="M25" s="1"/>
     </row>
@@ -2278,7 +2276,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>12</v>
@@ -2299,7 +2297,7 @@
         <v>1</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M26" s="1"/>
     </row>
@@ -2308,7 +2306,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>13</v>
@@ -2317,13 +2315,13 @@
         <v>5</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>1</v>
@@ -2335,7 +2333,7 @@
         <v>45952</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M27" s="1"/>
     </row>
@@ -2344,7 +2342,7 @@
         <v>1</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>13</v>
@@ -2353,13 +2351,13 @@
         <v>5</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>1</v>
@@ -2371,7 +2369,7 @@
         <v>45950</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M28" s="1"/>
     </row>
@@ -2380,7 +2378,7 @@
         <v>1</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>12</v>
@@ -2389,13 +2387,13 @@
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>1</v>
@@ -2407,7 +2405,7 @@
         <v>45930</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M29" s="1"/>
     </row>
@@ -2416,7 +2414,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>13</v>
@@ -2425,13 +2423,13 @@
         <v>6</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>1</v>
@@ -2443,7 +2441,7 @@
         <v>45954</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M30" s="1"/>
     </row>
@@ -2452,7 +2450,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>12</v>
@@ -2461,13 +2459,13 @@
         <v>0</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>1</v>
@@ -2476,7 +2474,7 @@
         <v>1</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M31" s="1"/>
     </row>
@@ -2485,7 +2483,7 @@
         <v>1</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>13</v>
@@ -2494,13 +2492,13 @@
         <v>6</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>1</v>
@@ -2509,7 +2507,7 @@
         <v>1</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M32" s="1"/>
     </row>
@@ -2518,7 +2516,7 @@
         <v>1</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>13</v>
@@ -2527,13 +2525,13 @@
         <v>6</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>1</v>
@@ -2542,7 +2540,7 @@
         <v>1</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M33" s="1"/>
     </row>
@@ -2551,7 +2549,7 @@
         <v>1</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>13</v>
@@ -2560,13 +2558,13 @@
         <v>6</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>1</v>
@@ -2578,7 +2576,7 @@
         <v>45954</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M34" s="1"/>
     </row>
@@ -2587,7 +2585,7 @@
         <v>1</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>12</v>
@@ -2596,13 +2594,13 @@
         <v>0</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>1</v>
@@ -2611,7 +2609,7 @@
         <v>1</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="M35" s="1"/>
     </row>
@@ -2620,7 +2618,7 @@
         <v>1</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>13</v>
@@ -2629,13 +2627,13 @@
         <v>5</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>1</v>
@@ -2644,7 +2642,7 @@
         <v>1</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M36" s="1"/>
     </row>
@@ -2653,7 +2651,7 @@
         <v>1</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>13</v>
@@ -2662,13 +2660,13 @@
         <v>5</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>1</v>
@@ -2677,7 +2675,7 @@
         <v>1</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="M37" s="1"/>
     </row>
@@ -2686,7 +2684,7 @@
         <v>1</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>13</v>
@@ -2695,13 +2693,13 @@
         <v>5</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>1</v>
@@ -2710,7 +2708,7 @@
         <v>1</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="M38" s="1"/>
     </row>
@@ -2719,7 +2717,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>13</v>
@@ -2728,13 +2726,13 @@
         <v>5</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>1</v>
@@ -2746,7 +2744,7 @@
         <v>45954</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M39" s="1"/>
     </row>
@@ -2755,7 +2753,7 @@
         <v>1</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>13</v>
@@ -2764,19 +2762,19 @@
         <v>5</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M40" s="1"/>
     </row>
@@ -2785,7 +2783,7 @@
         <v>1</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>12</v>
@@ -2794,13 +2792,13 @@
         <v>2</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>1</v>
@@ -2809,7 +2807,7 @@
         <v>1</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="M41" s="1"/>
     </row>
@@ -2818,7 +2816,7 @@
         <v>1</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>13</v>
@@ -2827,13 +2825,13 @@
         <v>7</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>1</v>
@@ -2842,7 +2840,7 @@
         <v>1</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M42" s="1"/>
     </row>
@@ -2851,7 +2849,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>12</v>
@@ -2860,13 +2858,13 @@
         <v>0</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>1</v>
@@ -2875,7 +2873,7 @@
         <v>1</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M43" s="1"/>
     </row>
@@ -2884,7 +2882,7 @@
         <v>1</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>12</v>
@@ -2893,13 +2891,13 @@
         <v>0</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>1</v>
@@ -2908,7 +2906,7 @@
         <v>1</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M44" s="1"/>
     </row>
@@ -2917,7 +2915,7 @@
         <v>1</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>13</v>
@@ -2926,13 +2924,13 @@
         <v>5</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>1</v>
@@ -2944,7 +2942,7 @@
         <v>46333</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M45" s="1"/>
     </row>
@@ -2953,7 +2951,7 @@
         <v>1</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>12</v>
@@ -2962,13 +2960,13 @@
         <v>0</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I46" s="1" t="s">
         <v>1</v>
@@ -2977,7 +2975,7 @@
         <v>1</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="M46" s="1"/>
     </row>
@@ -2986,7 +2984,7 @@
         <v>1</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>12</v>
@@ -2995,13 +2993,13 @@
         <v>0</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>1</v>
@@ -3010,7 +3008,7 @@
         <v>1</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M47" s="1"/>
     </row>
@@ -3019,7 +3017,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>12</v>
@@ -3028,13 +3026,13 @@
         <v>0</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>1</v>
@@ -3046,7 +3044,7 @@
         <v>45945</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M48" s="1"/>
     </row>
@@ -3055,7 +3053,7 @@
         <v>1</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>12</v>
@@ -3064,14 +3062,14 @@
         <v>0</v>
       </c>
       <c r="E49" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F49" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="G49" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="G49" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="I49" s="1" t="s">
         <v>1</v>
       </c>
@@ -3079,7 +3077,7 @@
         <v>1</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M49" s="1"/>
     </row>
@@ -3088,7 +3086,7 @@
         <v>1</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>12</v>
@@ -3097,13 +3095,13 @@
         <v>0</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>1</v>
@@ -3112,7 +3110,7 @@
         <v>1</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M50" s="1"/>
     </row>
@@ -3121,7 +3119,7 @@
         <v>1</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>13</v>
@@ -3130,13 +3128,13 @@
         <v>5</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>1</v>
@@ -3145,7 +3143,7 @@
         <v>1</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M51" s="1"/>
     </row>
@@ -3154,7 +3152,7 @@
         <v>1</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>13</v>
@@ -3163,13 +3161,13 @@
         <v>5</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I52" s="1" t="s">
         <v>1</v>
@@ -3178,7 +3176,7 @@
         <v>1</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M52" s="1"/>
     </row>
@@ -3187,7 +3185,7 @@
         <v>0</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>13</v>
@@ -3196,22 +3194,22 @@
         <v>5</v>
       </c>
       <c r="E53" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L53" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="I53" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="J53" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L53" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="M53" s="1"/>
     </row>
@@ -3220,7 +3218,7 @@
         <v>0</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>13</v>
@@ -3229,22 +3227,22 @@
         <v>5</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="J54" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M54" s="1"/>
     </row>
@@ -3253,7 +3251,7 @@
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>13</v>
@@ -3271,13 +3269,13 @@
         <v>8</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="J55" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M55" s="1"/>
     </row>
@@ -3286,7 +3284,7 @@
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>13</v>
@@ -3295,7 +3293,7 @@
         <v>6</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I56" s="1" t="s">
         <v>9</v>

</xml_diff>